<commit_message>
Add practice file for excel-001
</commit_message>
<xml_diff>
--- a/excel-001-practice.xlsx
+++ b/excel-001-practice.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="20">
   <si>
     <t xml:space="preserve">OrderID</t>
   </si>
@@ -37,34 +37,22 @@
     <t xml:space="preserve">Duplicate?</t>
   </si>
   <si>
-    <t xml:space="preserve">Summary</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chen Wei</t>
   </si>
   <si>
     <t xml:space="preserve">Berlin</t>
   </si>
   <si>
-    <t xml:space="preserve">Total rows</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hana Sato</t>
   </si>
   <si>
     <t xml:space="preserve">Toronto</t>
   </si>
   <si>
-    <t xml:space="preserve">Duplicate rows</t>
-  </si>
-  <si>
     <t xml:space="preserve">Elena Petrova</t>
   </si>
   <si>
     <t xml:space="preserve">Cairo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unique rows</t>
   </si>
   <si>
     <t xml:space="preserve">Grace Okafor</t>
@@ -98,10 +86,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -128,13 +117,6 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -197,7 +179,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -511,17 +493,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -540,31 +518,25 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
         <v>1001</v>
       </c>
       <c r="B2" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="2" t="n">
         <v>120</v>
       </c>
       <c r="E2" s="0" t="str">
         <f aca="false">IF(COUNTIF($A$2:A2,A2)&gt;1,"Duplicate","")</f>
         <v/>
       </c>
-      <c r="G2" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="0" t="n">
+      <c r="G2" s="0" t="n">
         <f aca="false">COUNTA(A2:A25)</f>
         <v>24</v>
       </c>
@@ -574,22 +546,19 @@
         <v>1003</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>870</v>
       </c>
       <c r="E3" s="0" t="str">
         <f aca="false">IF(COUNTIF($A$2:A3,A3)&gt;1,"Duplicate","")</f>
         <v/>
       </c>
-      <c r="G3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="0" t="n">
+      <c r="G3" s="0" t="n">
         <f aca="false">COUNTIF(E2:E25,"Duplicate")</f>
         <v>5</v>
       </c>
@@ -599,23 +568,20 @@
         <v>1018</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>465</v>
       </c>
       <c r="E4" s="0" t="str">
         <f aca="false">IF(COUNTIF($A$2:A4,A4)&gt;1,"Duplicate","")</f>
         <v/>
       </c>
-      <c r="G4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="0" t="n">
-        <f aca="false">H2-H3</f>
+      <c r="G4" s="0" t="n">
+        <f aca="false">G2-G3</f>
         <v>19</v>
       </c>
     </row>
@@ -624,17 +590,21 @@
         <v>1004</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>160</v>
       </c>
       <c r="E5" s="0" t="str">
         <f aca="false">IF(COUNTIF($A$2:A5,A5)&gt;1,"Duplicate","")</f>
         <v/>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">SUM(D2:D25)</f>
+        <v>10515</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -642,17 +612,21 @@
         <v>1005</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>535</v>
       </c>
       <c r="E6" s="0" t="str">
         <f aca="false">IF(COUNTIF($A$2:A6,A6)&gt;1,"Duplicate","")</f>
         <v/>
+      </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">SUMPRODUCT((E2:E25="")*D2:D25)</f>
+        <v>8015</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -660,12 +634,12 @@
         <v>1014</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>320</v>
       </c>
       <c r="E7" s="0" t="str">
@@ -678,12 +652,12 @@
         <v>1007</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>330</v>
       </c>
       <c r="E8" s="0" t="str">
@@ -696,12 +670,12 @@
         <v>1010</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="n">
         <v>525</v>
       </c>
       <c r="E9" s="0" t="str">
@@ -714,12 +688,12 @@
         <v>1018</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="n">
         <v>465</v>
       </c>
       <c r="E10" s="0" t="str">
@@ -732,12 +706,12 @@
         <v>1010</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="n">
         <v>525</v>
       </c>
       <c r="E11" s="0" t="str">
@@ -750,12 +724,12 @@
         <v>1015</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="D12" s="2" t="n">
         <v>65</v>
       </c>
       <c r="E12" s="0" t="str">
@@ -768,12 +742,12 @@
         <v>1011</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2" t="n">
         <v>75</v>
       </c>
       <c r="E13" s="0" t="str">
@@ -786,12 +760,12 @@
         <v>1012</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="n">
         <v>600</v>
       </c>
       <c r="E14" s="0" t="str">
@@ -804,12 +778,12 @@
         <v>1009</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="n">
         <v>70</v>
       </c>
       <c r="E15" s="0" t="str">
@@ -822,12 +796,12 @@
         <v>1007</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="D16" s="2" t="n">
         <v>330</v>
       </c>
       <c r="E16" s="0" t="str">
@@ -840,12 +814,12 @@
         <v>1006</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" s="2" t="n">
         <v>40</v>
       </c>
       <c r="E17" s="0" t="str">
@@ -858,12 +832,12 @@
         <v>1014</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>320</v>
       </c>
       <c r="E18" s="0" t="str">
@@ -876,12 +850,12 @@
         <v>1016</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="2" t="n">
         <v>860</v>
       </c>
       <c r="E19" s="0" t="str">
@@ -894,12 +868,12 @@
         <v>1008</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="n">
         <v>445</v>
       </c>
       <c r="E20" s="0" t="str">
@@ -912,12 +886,12 @@
         <v>1016</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="2" t="n">
         <v>860</v>
       </c>
       <c r="E21" s="0" t="str">
@@ -930,12 +904,12 @@
         <v>1002</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2" t="n">
         <v>670</v>
       </c>
       <c r="E22" s="0" t="str">
@@ -948,12 +922,12 @@
         <v>1019</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="2" t="n">
         <v>685</v>
       </c>
       <c r="E23" s="0" t="str">
@@ -966,12 +940,12 @@
         <v>1013</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="2" t="n">
         <v>335</v>
       </c>
       <c r="E24" s="0" t="str">
@@ -984,12 +958,12 @@
         <v>1017</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D25" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="2" t="n">
         <v>845</v>
       </c>
       <c r="E25" s="0" t="str">

</xml_diff>